<commit_message>
Add Pesto product monitoring category
</commit_message>
<xml_diff>
--- a/data/coles-woolworths-sauce-change-history.xlsx
+++ b/data/coles-woolworths-sauce-change-history.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,10 @@
       <color theme="10"/>
       <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="5">
@@ -89,7 +93,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -99,6 +103,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -594,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6687,12 +6692,89 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Pesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>Current Price (AUD)</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>Original Price (AUD)</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>Promotional Price (AUD)</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>Online Only</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="inlineStr">
+        <is>
+          <t>Availability</t>
+        </is>
+      </c>
+      <c r="J133" s="3" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="K133" s="3" t="inlineStr">
+        <is>
+          <t>Image URL</t>
+        </is>
+      </c>
+      <c r="L133" s="3" t="inlineStr">
+        <is>
+          <t>Product URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t>No matching SKUs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:L3"/>
+  <mergeCells count="5">
+    <mergeCell ref="A25:L25"/>
     <mergeCell ref="A107:L107"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A132:L132"/>
+    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
@@ -6951,7 +7033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12500,12 +12582,89 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Pesto</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Current Price (AUD)</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>Original Price (AUD)</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Promotional Price (AUD)</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>Online Only</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>Availability</t>
+        </is>
+      </c>
+      <c r="J123" s="3" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="K123" s="3" t="inlineStr">
+        <is>
+          <t>Image URL</t>
+        </is>
+      </c>
+      <c r="L123" s="3" t="inlineStr">
+        <is>
+          <t>Product URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t>No matching SKUs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A101:L101"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A122:L122"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
@@ -12767,87 +12926,87 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Observed (UTC)</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Retailer</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Before</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>After</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Current Price (AUD)</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Original Price (AUD)</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="8" t="inlineStr">
         <is>
           <t>Promotional Price (AUD)</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="8" t="inlineStr">
         <is>
           <t>Discount</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Online Only</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Availability</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="O1" s="8" t="inlineStr">
         <is>
           <t>Image URL</t>
         </is>
       </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="P1" s="8" t="inlineStr">
         <is>
           <t>Product URL</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="Q1" s="8" t="inlineStr">
         <is>
           <t>Event ID</t>
         </is>

</xml_diff>

<commit_message>
Capture multibuy offers and simplify SKU changes
</commit_message>
<xml_diff>
--- a/data/coles-woolworths-sauce-change-history.xlsx
+++ b/data/coles-woolworths-sauce-change-history.xlsx
@@ -260,8 +260,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="WoolworthsTomatoPasteTable" displayName="WoolworthsTomatoPasteTable" ref="A4:K23" headerRowCount="1">
-  <autoFilter ref="A4:K23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="WoolworthsTomatoPasteTable" displayName="WoolworthsTomatoPasteTable" ref="A4:K22" headerRowCount="1">
+  <autoFilter ref="A4:K22"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Product ID"/>
     <tableColumn id="2" name="Brand"/>
@@ -280,8 +280,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="WoolworthsPastaSauceTable" displayName="WoolworthsPastaSauceTable" ref="A26:K98" headerRowCount="1">
-  <autoFilter ref="A26:K98"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="WoolworthsPastaSauceTable" displayName="WoolworthsPastaSauceTable" ref="A25:K98" headerRowCount="1">
+  <autoFilter ref="A25:K98"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Product ID"/>
     <tableColumn id="2" name="Brand"/>
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="WoolworthsPassataTable" displayName="WoolworthsPassataTable" ref="A101:K119" headerRowCount="1">
-  <autoFilter ref="A101:K119"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="WoolworthsPassataTable" displayName="WoolworthsPassataTable" ref="A101:K121" headerRowCount="1">
+  <autoFilter ref="A101:K121"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Product ID"/>
     <tableColumn id="2" name="Brand"/>
@@ -320,8 +320,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="WoolworthsPestoTable" displayName="WoolworthsPestoTable" ref="A122:K141" headerRowCount="1">
-  <autoFilter ref="A122:K141"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="WoolworthsPestoTable" displayName="WoolworthsPestoTable" ref="A124:K144" headerRowCount="1">
+  <autoFilter ref="A124:K144"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Product ID"/>
     <tableColumn id="2" name="Brand"/>
@@ -6641,7 +6641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K141"/>
+  <dimension ref="A1:K144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6774,7 +6774,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>woolworths:22078</t>
+          <t>woolworths:85045</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6788,7 +6788,7 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>3.5</v>
+        <v>4.8</v>
       </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
@@ -6805,19 +6805,19 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>140g x 2 pack</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/22078/leggo-s-australian-grown-tomato-paste-no-added-salt</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/85045/leggo-s-australian-grown-tomato-paste-no-added-salt</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>woolworths:85045</t>
+          <t>woolworths:22078</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6831,7 +6831,7 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>4.8</v>
+        <v>3.5</v>
       </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
@@ -6848,12 +6848,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>140g x 2 pack</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/85045/leggo-s-australian-grown-tomato-paste-no-added-salt</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/22078/leggo-s-australian-grown-tomato-paste-no-added-salt</t>
         </is>
       </c>
     </row>
@@ -7167,7 +7167,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>woolworths:290303</t>
+          <t>woolworths:81641</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7181,16 +7181,16 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>1.65</v>
+        <v>2.8</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>2.4</v>
+        <v>4</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>1.65</v>
+        <v>2.8</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0.3125</v>
+        <v>0.3</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -7204,19 +7204,19 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>130g</t>
+          <t>140g x 2 pack</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/290303/mutti-tomato-paste-double-concentrate</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/81641/mutti-tomato-paste-double-concentrate</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>woolworths:81641</t>
+          <t>woolworths:290303</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7230,16 +7230,16 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>2.8</v>
+        <v>1.65</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>2.8</v>
+        <v>1.65</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0.3</v>
+        <v>0.3125</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -7253,12 +7253,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>140g x 2 pack</t>
+          <t>130g</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/81641/mutti-tomato-paste-double-concentrate</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/290303/mutti-tomato-paste-double-concentrate</t>
         </is>
       </c>
     </row>
@@ -7308,21 +7308,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>woolworths:194802</t>
+          <t>woolworths:90260</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tukas</t>
+          <t>Woolworths Essentials</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Tukas Tomato Paste Jar</t>
+          <t>Woolworths Essentials Tomato Paste</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>6.2</v>
+        <v>0.95</v>
       </c>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
@@ -7339,12 +7339,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>700g</t>
+          <t>170g</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/194802/tukas-tomato-paste-jar</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/90260/woolworths-essentials-tomato-paste</t>
         </is>
       </c>
     </row>
@@ -7394,21 +7394,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>woolworths:90260</t>
+          <t>woolworths:258476</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Woolworths Essentials</t>
+          <t>Woolworths</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Woolworths Essentials Tomato Paste</t>
+          <t>Woolworths Tomato Paste</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.95</v>
+        <v>2.5</v>
       </c>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
@@ -7425,19 +7425,19 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>170g</t>
+          <t>415g</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/90260/woolworths-essentials-tomato-paste</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/258476/woolworths-tomato-paste</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>woolworths:258476</t>
+          <t>woolworths:748896</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7447,11 +7447,11 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Woolworths Tomato Paste</t>
+          <t>Woolworths Tomato Paste Sachet</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>2.5</v>
+        <v>2.35</v>
       </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
@@ -7468,19 +7468,19 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>415g</t>
+          <t>4 pack</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/258476/woolworths-tomato-paste</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/748896/woolworths-tomato-paste-sachet</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>woolworths:748896</t>
+          <t>woolworths:197787</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Woolworths Tomato Paste Sachet</t>
+          <t>Woolworths Tomato Paste Sachets No Added Salt</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
@@ -7516,133 +7516,135 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/748896/woolworths-tomato-paste-sachet</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>woolworths:197787</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Woolworths</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Woolworths Tomato Paste Sachets No Added Salt</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Temporarily unavailable</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>4 pack</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
           <t>https://www.woolworths.com.au/shop/productdetails/197787/woolworths-tomato-paste-sachets-no-added-salt</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Pasta Sauce</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Pasta Sauce</t>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Product ID</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Current Price (AUD)</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Original Price (AUD)</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Promotional Price (AUD)</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Online Only</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Availability</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Product URL</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Product ID</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Current Price (AUD)</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Original Price (AUD)</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Promotional Price (AUD)</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Discount</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Online Only</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>Availability</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>Size</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>Product URL</t>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>woolworths:76670</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Artisanology</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Artisanology Truffle Pasta Sauce</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>450g</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://www.woolworths.com.au/shop/productdetails/76670/artisanology-truffle-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>woolworths:78934</t>
+          <t>woolworths:504885</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Aurelio</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Barilla Arrabbiata Pasta Sauce Arrabbiata Chilli</t>
+          <t>Aurelio Arribiatta Organic Pasta Sauce</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>3.6</v>
+        <v>6</v>
       </c>
       <c r="E27" s="5" t="n"/>
       <c r="F27" s="5" t="n"/>
@@ -7659,33 +7661,33 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/78934/barilla-arrabbiata-pasta-sauce-arrabbiata-chilli</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/504885/aurelio-arribiatta-organic-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>woolworths:190944</t>
+          <t>woolworths:504884</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Aurelio</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Barilla Basil Pesto Vegan Pasta Sauce</t>
+          <t>Aurelio Basillico Organic Pasta Sauce</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="E28" s="5" t="n"/>
       <c r="F28" s="5" t="n"/>
@@ -7702,19 +7704,19 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>190g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/190944/barilla-basil-pesto-vegan-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/504884/aurelio-basillico-organic-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>woolworths:78921</t>
+          <t>woolworths:78934</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7724,7 +7726,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Barilla Basilico Pasta Sauce Basilico Tomato Basil</t>
+          <t>Barilla Arrabbiata Pasta Sauce Arrabbiata Chilli</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
@@ -7750,14 +7752,14 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/78921/barilla-basilico-pasta-sauce-basilico-tomato-basil</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/78934/barilla-arrabbiata-pasta-sauce-arrabbiata-chilli</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>woolworths:315578</t>
+          <t>woolworths:190944</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7767,11 +7769,11 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Barilla Bolognese Pasta Sauce Bolognese</t>
+          <t>Barilla Basil Pesto Vegan Pasta Sauce</t>
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>3.6</v>
+        <v>5.3</v>
       </c>
       <c r="E30" s="5" t="n"/>
       <c r="F30" s="5" t="n"/>
@@ -7788,19 +7790,19 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>190g</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/315578/barilla-bolognese-pasta-sauce-bolognese</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/190944/barilla-basil-pesto-vegan-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>woolworths:146359</t>
+          <t>woolworths:78921</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7810,7 +7812,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Barilla Napoletana Pasta Sauce Napoletana</t>
+          <t>Barilla Basilico Pasta Sauce Basilico Tomato Basil</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
@@ -7836,14 +7838,14 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/146359/barilla-napoletana-pasta-sauce-napoletana</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/78921/barilla-basilico-pasta-sauce-basilico-tomato-basil</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>woolworths:3466</t>
+          <t>woolworths:315578</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7853,11 +7855,11 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Barilla Pesto Genovese Pasta Sauce Alla Genovese</t>
+          <t>Barilla Bolognese Pasta Sauce Bolognese</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>5.3</v>
+        <v>3.6</v>
       </c>
       <c r="E32" s="5" t="n"/>
       <c r="F32" s="5" t="n"/>
@@ -7874,19 +7876,19 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>190g</t>
+          <t>400g</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/3466/barilla-pesto-genovese-pasta-sauce-alla-genovese</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/315578/barilla-bolognese-pasta-sauce-bolognese</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>woolworths:238030</t>
+          <t>woolworths:146359</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7896,11 +7898,11 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Barilla Pesto Rosso Pasta Sauce</t>
+          <t>Barilla Napoletana Pasta Sauce Napoletana</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>5.9</v>
+        <v>3.6</v>
       </c>
       <c r="E33" s="5" t="n"/>
       <c r="F33" s="5" t="n"/>
@@ -7917,43 +7919,37 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>200g</t>
+          <t>400g</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/238030/barilla-pesto-rosso-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/146359/barilla-napoletana-pasta-sauce-napoletana</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>woolworths:6040643</t>
+          <t>woolworths:3466</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bella Cucina</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Bella Cucina Alla Vodka Pasta Sauce</t>
+          <t>Barilla Pesto Genovese Pasta Sauce Alla Genovese</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E34" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F34" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G34" s="6" t="n">
-        <v>0.5</v>
-      </c>
+        <v>5.3</v>
+      </c>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="6" t="n"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>No</t>
@@ -7966,43 +7962,37 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>190g</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6040643/bella-cucina-alla-vodka-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/3466/barilla-pesto-genovese-pasta-sauce-alla-genovese</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>woolworths:6040753</t>
+          <t>woolworths:238030</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Bella Cucina</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Bella Cucina Arrabbiata Pasta Sauce</t>
+          <t>Barilla Pesto Rosso Pasta Sauce</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E35" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F35" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G35" s="6" t="n">
-        <v>0.5</v>
-      </c>
+        <v>5.9</v>
+      </c>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="6" t="n"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>No</t>
@@ -8015,32 +8005,34 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>200g</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6040753/bella-cucina-arrabbiata-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/238030/barilla-pesto-rosso-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>woolworths:6040684</t>
+          <t>woolworths:758377</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bella Cucina</t>
+          <t>Dolmio</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Bella Cucina Basil Sugo Pasta Sauce</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="n"/>
+          <t>Dolmio Classic Tomato With Basil Pasta Sauce</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>2.5</v>
+      </c>
       <c r="E36" s="5" t="n"/>
       <c r="F36" s="5" t="n"/>
       <c r="G36" s="6" t="n"/>
@@ -8051,48 +8043,42 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Temporarily unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6040684/bella-cucina-basil-sugo-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/758377/dolmio-classic-tomato-with-basil-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>woolworths:6040682</t>
+          <t>woolworths:758447</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Bella Cucina</t>
+          <t>Dolmio</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Bella Cucina Passata Pasta Sauce</t>
+          <t>Dolmio Creamy Carbonara Pasta Sauce</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F37" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>0.5</v>
-      </c>
+        <v>4.6</v>
+      </c>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="6" t="n"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>No</t>
@@ -8105,43 +8091,37 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>490g</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6040682/bella-cucina-passata-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/758447/dolmio-creamy-carbonara-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>woolworths:6040823</t>
+          <t>woolworths:758286</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bella Cucina</t>
+          <t>Dolmio</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Bella Cucina Pomodoro Pasta Sauce</t>
+          <t>Dolmio Extra Bolognese Tomato Pasta Sauce</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E38" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G38" s="6" t="n">
-        <v>0.5</v>
-      </c>
+        <v>4.6</v>
+      </c>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="6" t="n"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>No</t>
@@ -8154,19 +8134,19 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6040823/bella-cucina-pomodoro-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/758286/dolmio-extra-bolognese-tomato-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>woolworths:758377</t>
+          <t>woolworths:758288</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8176,11 +8156,11 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Dolmio Classic Tomato With Basil Pasta Sauce</t>
+          <t>Dolmio Extra Red Wine &amp; Italian Herbs Tomato Pasta Sauce</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>2.5</v>
+        <v>4.6</v>
       </c>
       <c r="E39" s="5" t="n"/>
       <c r="F39" s="5" t="n"/>
@@ -8202,14 +8182,14 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/758377/dolmio-classic-tomato-with-basil-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/758288/dolmio-extra-red-wine-italian-herbs-tomato-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>woolworths:758447</t>
+          <t>woolworths:758299</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8219,7 +8199,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Dolmio Creamy Carbonara Pasta Sauce</t>
+          <t>Dolmio Extra Spicy Peppers Tomato Pasta Sauce</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
@@ -8240,19 +8220,19 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>490g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/758447/dolmio-creamy-carbonara-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/758299/dolmio-extra-spicy-peppers-tomato-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>woolworths:758286</t>
+          <t>woolworths:758342</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8262,7 +8242,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Dolmio Extra Bolognese Tomato Pasta Sauce</t>
+          <t>Dolmio Extra Tomato Onion &amp; Roast Garlic Pasta Sauce</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
@@ -8288,28 +8268,28 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/758286/dolmio-extra-bolognese-tomato-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/758342/dolmio-extra-tomato-onion-roast-garlic-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>woolworths:758288</t>
+          <t>woolworths:963209</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dolmio</t>
+          <t>Don Antonio</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Dolmio Extra Red Wine &amp; Italian Herbs Tomato Pasta Sauce</t>
+          <t>Don Antonio Pasta Sauce Sugo Al Basilico</t>
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>4.6</v>
+        <v>7</v>
       </c>
       <c r="E42" s="5" t="n"/>
       <c r="F42" s="5" t="n"/>
@@ -8331,28 +8311,28 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/758288/dolmio-extra-red-wine-italian-herbs-tomato-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/963209/don-antonio-pasta-sauce-sugo-al-basilico</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>woolworths:758299</t>
+          <t>woolworths:647692</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dolmio</t>
+          <t>Fodmapped For You</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Dolmio Extra Spicy Peppers Tomato Pasta Sauce</t>
+          <t>Fodmapped For You Red Wine &amp; Italian Herbs Tomato Pasta Sauce</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>4.6</v>
+        <v>6.5</v>
       </c>
       <c r="E43" s="5" t="n"/>
       <c r="F43" s="5" t="n"/>
@@ -8369,33 +8349,33 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>375g</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/758299/dolmio-extra-spicy-peppers-tomato-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/647692/fodmapped-for-you-red-wine-italian-herbs-tomato-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>woolworths:758342</t>
+          <t>woolworths:149303</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dolmio</t>
+          <t>Fodmapped For You</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Dolmio Extra Tomato Onion &amp; Roast Garlic Pasta Sauce</t>
+          <t>Fodmapped For You Tomato Pasta Sauce Bolognaise</t>
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>4.6</v>
+        <v>6.5</v>
       </c>
       <c r="E44" s="5" t="n"/>
       <c r="F44" s="5" t="n"/>
@@ -8412,33 +8392,33 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>375g</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/758342/dolmio-extra-tomato-onion-roast-garlic-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/149303/fodmapped-for-you-tomato-pasta-sauce-bolognaise</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>woolworths:963209</t>
+          <t>woolworths:34057</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Don Antonio</t>
+          <t>Heinz</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Don Antonio Pasta Sauce Sugo Al Basilico</t>
+          <t>Heinz Canned Spaghetti Pasta In Tomato Sauce</t>
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>7</v>
+        <v>2.1</v>
       </c>
       <c r="E45" s="5" t="n"/>
       <c r="F45" s="5" t="n"/>
@@ -8455,33 +8435,29 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>220g</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/963209/don-antonio-pasta-sauce-sugo-al-basilico</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/34057/heinz-canned-spaghetti-pasta-in-tomato-sauce</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>woolworths:647692</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Fodmapped For You</t>
-        </is>
-      </c>
+          <t>woolworths:1125367633</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Fodmapped For You Red Wine &amp; Italian Herbs Tomato Pasta Sauce</t>
+          <t>Kitchen Cooking Splash Guard - Frying Pasta Sauce Curry Anti Splatter Screen Shield - Oil Grease Splatter</t>
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>6.5</v>
+        <v>21.95</v>
       </c>
       <c r="E46" s="5" t="n"/>
       <c r="F46" s="5" t="n"/>
@@ -8496,36 +8472,30 @@
           <t>Available</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>375g</t>
-        </is>
-      </c>
+      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/647692/fodmapped-for-you-red-wine-italian-herbs-tomato-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/1125367633/kitchen-cooking-splash-guard-frying-pasta-sauce-curry-anti-splatter-screen-shield-oil-grease-splatter</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>woolworths:149303</t>
+          <t>woolworths:6023653</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Fodmapped For You</t>
+          <t>La Gina</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Fodmapped For You Tomato Pasta Sauce Bolognaise</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="n">
-        <v>6.5</v>
-      </c>
+          <t>La Gina Bolognese Pasta Sauce</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="n"/>
       <c r="E47" s="5" t="n"/>
       <c r="F47" s="5" t="n"/>
       <c r="G47" s="6" t="n"/>
@@ -8536,38 +8506,38 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Temporarily unavailable</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>375g</t>
+          <t>400g</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/149303/fodmapped-for-you-tomato-pasta-sauce-bolognaise</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6023653/la-gina-bolognese-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>woolworths:34057</t>
+          <t>woolworths:6023655</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Heinz</t>
+          <t>La Gina</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Heinz Canned Spaghetti Pasta In Tomato Sauce</t>
+          <t>La Gina Calabrese Pasta Sauce</t>
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>2.1</v>
+        <v>4</v>
       </c>
       <c r="E48" s="5" t="n"/>
       <c r="F48" s="5" t="n"/>
@@ -8584,29 +8554,33 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>220g</t>
+          <t>400g</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/34057/heinz-canned-spaghetti-pasta-in-tomato-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6023655/la-gina-calabrese-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>woolworths:1125367633</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
+          <t>woolworths:6023652</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>La Gina</t>
+        </is>
+      </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Kitchen Cooking Splash Guard - Frying Pasta Sauce Curry Anti Splatter Screen Shield - Oil Grease Splatter</t>
+          <t>La Gina Siciliana Pasta Sauce</t>
         </is>
       </c>
       <c r="D49" s="5" t="n">
-        <v>21.95</v>
+        <v>4</v>
       </c>
       <c r="E49" s="5" t="n"/>
       <c r="F49" s="5" t="n"/>
@@ -8621,27 +8595,31 @@
           <t>Available</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>400g</t>
+        </is>
+      </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/1125367633/kitchen-cooking-splash-guard-frying-pasta-sauce-curry-anti-splatter-screen-shield-oil-grease-splatter</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6023652/la-gina-siciliana-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>woolworths:6023653</t>
+          <t>woolworths:6024441</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>La Gina</t>
+          <t>La Tosca</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>La Gina Bolognese Pasta Sauce</t>
+          <t>La Tosca Napoletana Pasta Sauce</t>
         </is>
       </c>
       <c r="D50" s="5" t="n">
@@ -8662,33 +8640,33 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>425g</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6023653/la-gina-bolognese-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6024441/la-tosca-napoletana-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>woolworths:6023655</t>
+          <t>woolworths:321163</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>La Gina</t>
+          <t>Leggo's</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>La Gina Calabrese Pasta Sauce</t>
+          <t>Leggo's Bacon Flavour Bolognese Chunky Tomato &amp; Herbs Pasta Sauce</t>
         </is>
       </c>
       <c r="D51" s="5" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="E51" s="5" t="n"/>
       <c r="F51" s="5" t="n"/>
@@ -8705,33 +8683,33 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6023655/la-gina-calabrese-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/321163/leggo-s-bacon-flavour-bolognese-chunky-tomato-herbs-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>woolworths:6023652</t>
+          <t>woolworths:6058442</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>La Gina</t>
+          <t>Leggo's</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>La Gina Siciliana Pasta Sauce</t>
+          <t>Leggo's Beef Ragu with Chunky Tomato Garlic &amp; Herbs Pasta Sauce</t>
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="E52" s="5" t="n"/>
       <c r="F52" s="5" t="n"/>
@@ -8748,33 +8726,33 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6023652/la-gina-siciliana-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6058442/leggo-s-beef-ragu-with-chunky-tomato-garlic-herbs-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>woolworths:6024441</t>
+          <t>woolworths:450687</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>La Tosca</t>
+          <t>Leggo's</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>La Tosca Napoletana Pasta Sauce</t>
+          <t>Leggo's Bolognese Chunky Tomato Garlic &amp; Herbs Pasta Sauce</t>
         </is>
       </c>
       <c r="D53" s="5" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="E53" s="5" t="n"/>
       <c r="F53" s="5" t="n"/>
@@ -8791,19 +8769,19 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>425g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6024441/la-tosca-napoletana-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/450687/leggo-s-bolognese-chunky-tomato-garlic-herbs-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>woolworths:321163</t>
+          <t>woolworths:6038784</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8813,7 +8791,7 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Bacon Flavour Bolognese Chunky Tomato &amp; Herbs Pasta Sauce</t>
+          <t>Leggo's Creamy Carbonara Pasta Sauce</t>
         </is>
       </c>
       <c r="D54" s="5" t="n">
@@ -8834,19 +8812,19 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>490g</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/321163/leggo-s-bacon-flavour-bolognese-chunky-tomato-herbs-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6038784/leggo-s-creamy-carbonara-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>woolworths:6058442</t>
+          <t>woolworths:452061</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8856,11 +8834,11 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Beef Ragu with Chunky Tomato Garlic &amp; Herbs Pasta Sauce</t>
+          <t>Leggo's Creamy Sundried Tomato &amp; Garlic Pasta Bake Sauce</t>
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="E55" s="5" t="n"/>
       <c r="F55" s="5" t="n"/>
@@ -8882,14 +8860,14 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6058442/leggo-s-beef-ragu-with-chunky-tomato-garlic-herbs-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/452061/leggo-s-creamy-sundried-tomato-garlic-pasta-bake-sauce</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>woolworths:450687</t>
+          <t>woolworths:680702</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8899,11 +8877,11 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Bolognese Chunky Tomato Garlic &amp; Herbs Pasta Sauce</t>
+          <t>Leggo's Creamy Three Cheese Pasta Bake Sauce</t>
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="E56" s="5" t="n"/>
       <c r="F56" s="5" t="n"/>
@@ -8925,14 +8903,14 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/450687/leggo-s-bolognese-chunky-tomato-garlic-herbs-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/680702/leggo-s-creamy-three-cheese-pasta-bake-sauce</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>woolworths:6038784</t>
+          <t>woolworths:452050</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8942,11 +8920,11 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Creamy Carbonara Pasta Sauce</t>
+          <t>Leggo's Creamy Tomato &amp; Mozzarella Pasta Bake Sauce</t>
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="E57" s="5" t="n"/>
       <c r="F57" s="5" t="n"/>
@@ -8963,19 +8941,19 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>490g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6038784/leggo-s-creamy-carbonara-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/452050/leggo-s-creamy-tomato-mozzarella-pasta-bake-sauce</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>woolworths:452061</t>
+          <t>woolworths:6058427</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8985,15 +8963,21 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Creamy Sundried Tomato &amp; Garlic Pasta Bake Sauce</t>
+          <t>Leggo's Gourmet Cacio e Pepe Pasta Sauce</t>
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="E58" s="5" t="n"/>
-      <c r="F58" s="5" t="n"/>
-      <c r="G58" s="6" t="n"/>
+        <v>3.8</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F58" s="5" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>0.2083</v>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>No</t>
@@ -9006,19 +8990,19 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>390g</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/452061/leggo-s-creamy-sundried-tomato-garlic-pasta-bake-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6058427/leggo-s-gourmet-cacio-e-pepe-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>woolworths:680702</t>
+          <t>woolworths:6039158</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -9028,15 +9012,21 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Creamy Three Cheese Pasta Bake Sauce</t>
+          <t>Leggo's Gourmet Tomato &amp; Adelaide Hills Chardonnay Pasta Sauce</t>
         </is>
       </c>
       <c r="D59" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="E59" s="5" t="n"/>
-      <c r="F59" s="5" t="n"/>
-      <c r="G59" s="6" t="n"/>
+        <v>3.8</v>
+      </c>
+      <c r="E59" s="5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F59" s="5" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>0.2083</v>
+      </c>
       <c r="H59" t="inlineStr">
         <is>
           <t>No</t>
@@ -9049,19 +9039,19 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>390g</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/680702/leggo-s-creamy-three-cheese-pasta-bake-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6039158/leggo-s-gourmet-tomato-adelaide-hills-chardonnay-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>woolworths:452050</t>
+          <t>woolworths:317353</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -9071,15 +9061,21 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Creamy Tomato &amp; Mozzarella Pasta Bake Sauce</t>
+          <t>Leggo's Gourmet Tomato &amp; Pepperjack Shiraz Pasta Sauce</t>
         </is>
       </c>
       <c r="D60" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="E60" s="5" t="n"/>
-      <c r="F60" s="5" t="n"/>
-      <c r="G60" s="6" t="n"/>
+        <v>3.8</v>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F60" s="5" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="G60" s="6" t="n">
+        <v>0.2083</v>
+      </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>No</t>
@@ -9092,19 +9088,19 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>390g</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/452050/leggo-s-creamy-tomato-mozzarella-pasta-bake-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/317353/leggo-s-gourmet-tomato-pepperjack-shiraz-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>woolworths:6058427</t>
+          <t>woolworths:6038814</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -9114,7 +9110,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Gourmet Cacio e Pepe Pasta Sauce</t>
+          <t>Leggo's Gourmet Tomato &amp; Umami Papi Chilli Oil Pasta Sauce</t>
         </is>
       </c>
       <c r="D61" s="5" t="n">
@@ -9146,14 +9142,14 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6058427/leggo-s-gourmet-cacio-e-pepe-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6038814/leggo-s-gourmet-tomato-umami-papi-chilli-oil-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>woolworths:6039158</t>
+          <t>woolworths:6058426</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -9163,21 +9159,15 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Gourmet Tomato &amp; Adelaide Hills Chardonnay Pasta Sauce</t>
+          <t>Leggo's Marry Me Chicken Pasta Bake Sauce</t>
         </is>
       </c>
       <c r="D62" s="5" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="E62" s="5" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="F62" s="5" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="G62" s="6" t="n">
-        <v>0.2083</v>
-      </c>
+        <v>4.3</v>
+      </c>
+      <c r="E62" s="5" t="n"/>
+      <c r="F62" s="5" t="n"/>
+      <c r="G62" s="6" t="n"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>No</t>
@@ -9190,19 +9180,19 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>390g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6039158/leggo-s-gourmet-tomato-adelaide-hills-chardonnay-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6058426/leggo-s-marry-me-chicken-pasta-bake-sauce</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>woolworths:317353</t>
+          <t>woolworths:451926</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -9212,21 +9202,15 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Gourmet Tomato &amp; Pepperjack Shiraz Pasta Sauce</t>
+          <t>Leggo's Mushroom Bolognese With Chunky Tomato &amp; Herbs Pasta Sauce</t>
         </is>
       </c>
       <c r="D63" s="5" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="E63" s="5" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="F63" s="5" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="G63" s="6" t="n">
-        <v>0.2083</v>
-      </c>
+        <v>3.3</v>
+      </c>
+      <c r="E63" s="5" t="n"/>
+      <c r="F63" s="5" t="n"/>
+      <c r="G63" s="6" t="n"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>No</t>
@@ -9239,19 +9223,19 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>390g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/317353/leggo-s-gourmet-tomato-pepperjack-shiraz-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/451926/leggo-s-mushroom-bolognese-with-chunky-tomato-herbs-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>woolworths:6038814</t>
+          <t>woolworths:450822</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -9261,21 +9245,15 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Gourmet Tomato &amp; Umami Papi Chilli Oil Pasta Sauce</t>
+          <t>Leggo's Napoletana With Chunky Tomato &amp; Herbs Pasta Sauce</t>
         </is>
       </c>
       <c r="D64" s="5" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="E64" s="5" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="F64" s="5" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="G64" s="6" t="n">
-        <v>0.2083</v>
-      </c>
+        <v>3.3</v>
+      </c>
+      <c r="E64" s="5" t="n"/>
+      <c r="F64" s="5" t="n"/>
+      <c r="G64" s="6" t="n"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>No</t>
@@ -9288,19 +9266,19 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>390g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6038814/leggo-s-gourmet-tomato-umami-papi-chilli-oil-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/450822/leggo-s-napoletana-with-chunky-tomato-herbs-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>woolworths:6058426</t>
+          <t>woolworths:38648</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -9310,11 +9288,11 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Marry Me Chicken Pasta Bake Sauce</t>
+          <t>Leggo's Pasta Sauce Spaghetti With Beef</t>
         </is>
       </c>
       <c r="D65" s="5" t="n">
-        <v>4.3</v>
+        <v>5</v>
       </c>
       <c r="E65" s="5" t="n"/>
       <c r="F65" s="5" t="n"/>
@@ -9331,19 +9309,19 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>500g</t>
+          <t>680g</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6058426/leggo-s-marry-me-chicken-pasta-bake-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/38648/leggo-s-pasta-sauce-spaghetti-with-beef</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>woolworths:451926</t>
+          <t>woolworths:451922</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -9353,7 +9331,7 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Mushroom Bolognese With Chunky Tomato &amp; Herbs Pasta Sauce</t>
+          <t>Leggo's Red Wine Bolognese With Chunky Tomato &amp; Herbs Pasta Sauce</t>
         </is>
       </c>
       <c r="D66" s="5" t="n">
@@ -9379,14 +9357,14 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/451926/leggo-s-mushroom-bolognese-with-chunky-tomato-herbs-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/451922/leggo-s-red-wine-bolognese-with-chunky-tomato-herbs-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>woolworths:450822</t>
+          <t>woolworths:451923</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -9396,7 +9374,7 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Napoletana With Chunky Tomato &amp; Herbs Pasta Sauce</t>
+          <t>Leggo's Roasted Garlic Chunky Tomato &amp; Onion Pasta Sauce</t>
         </is>
       </c>
       <c r="D67" s="5" t="n">
@@ -9422,14 +9400,14 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/450822/leggo-s-napoletana-with-chunky-tomato-herbs-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/451923/leggo-s-roasted-garlic-chunky-tomato-onion-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>woolworths:38648</t>
+          <t>woolworths:452031</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -9439,11 +9417,11 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Pasta Sauce Spaghetti With Beef</t>
+          <t>Leggo's Tuna Bake Pasta Sauce</t>
         </is>
       </c>
       <c r="D68" s="5" t="n">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="E68" s="5" t="n"/>
       <c r="F68" s="5" t="n"/>
@@ -9460,37 +9438,45 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>680g</t>
+          <t>500g</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/38648/leggo-s-pasta-sauce-spaghetti-with-beef</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/452031/leggo-s-tuna-bake-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>woolworths:451922</t>
+          <t>woolworths:348403</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Leggo's</t>
+          <t>Lucia's</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Red Wine Bolognese With Chunky Tomato &amp; Herbs Pasta Sauce</t>
+          <t>Lucia's Arrabbiata Pasta Sauce Arrabbiata Pasta Sauce</t>
         </is>
       </c>
       <c r="D69" s="5" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="E69" s="5" t="n"/>
-      <c r="F69" s="5" t="n"/>
-      <c r="G69" s="6" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="E69" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>2 for $14.00</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="n">
+        <v>0.125</v>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>No</t>
@@ -9508,32 +9494,40 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/451922/leggo-s-red-wine-bolognese-with-chunky-tomato-herbs-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/348403/lucia-s-arrabbiata-pasta-sauce-arrabbiata-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>woolworths:451923</t>
+          <t>woolworths:303965</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Leggo's</t>
+          <t>Lucia's</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Roasted Garlic Chunky Tomato &amp; Onion Pasta Sauce</t>
+          <t>Lucia's Napoletana Pasta Sauce Napoletana Pasta Sauce</t>
         </is>
       </c>
       <c r="D70" s="5" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="E70" s="5" t="n"/>
-      <c r="F70" s="5" t="n"/>
-      <c r="G70" s="6" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="E70" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>2 for $14.00</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="n">
+        <v>0.125</v>
+      </c>
       <c r="H70" t="inlineStr">
         <is>
           <t>No</t>
@@ -9551,32 +9545,40 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/451923/leggo-s-roasted-garlic-chunky-tomato-onion-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/303965/lucia-s-napoletana-pasta-sauce-napoletana-pasta-sauce</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>woolworths:452031</t>
+          <t>woolworths:200698</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Leggo's</t>
+          <t>Lucia's</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Tuna Bake Pasta Sauce</t>
+          <t>Lucia's Tomatoes &amp; Basil Pasta Sauce Tomatoes &amp; Basil Pasta Sauce</t>
         </is>
       </c>
       <c r="D71" s="5" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="E71" s="5" t="n"/>
-      <c r="F71" s="5" t="n"/>
-      <c r="G71" s="6" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="E71" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>2 for $14.00</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="n">
+        <v>0.125</v>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>No</t>
@@ -9594,7 +9596,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/452031/leggo-s-tuna-bake-pasta-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/200698/lucia-s-tomatoes-basil-pasta-sauce-tomatoes-basil-pasta-sauce</t>
         </is>
       </c>
     </row>
@@ -11321,22 +11323,20 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>woolworths:700648</t>
+          <t>woolworths:303969</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Macro</t>
+          <t>Lucia's</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Macro Organic Passata</t>
-        </is>
-      </c>
-      <c r="D111" s="5" t="n">
-        <v>2.5</v>
-      </c>
+          <t>Lucia's Passata Sauce Passata Sauce</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="n"/>
       <c r="E111" s="5" t="n"/>
       <c r="F111" s="5" t="n"/>
       <c r="G111" s="6" t="n"/>
@@ -11347,7 +11347,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Temporarily unavailable</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -11357,38 +11357,32 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/700648/macro-organic-passata</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/303969/lucia-s-passata-sauce-passata-sauce</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>woolworths:81719</t>
+          <t>woolworths:700648</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Mutti</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Mutti Baby Roma Passata Tomato Puree Gastronomia</t>
+          <t>Macro Organic Passata</t>
         </is>
       </c>
       <c r="D112" s="5" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="E112" s="5" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="F112" s="5" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="G112" s="6" t="n">
-        <v>0.3085</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="E112" s="5" t="n"/>
+      <c r="F112" s="5" t="n"/>
+      <c r="G112" s="6" t="n"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>No</t>
@@ -11401,19 +11395,19 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>700g</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/81719/mutti-baby-roma-passata-tomato-puree-gastronomia</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/700648/macro-organic-passata</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>woolworths:81718</t>
+          <t>woolworths:81719</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -11423,7 +11417,7 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Mutti Cherry Tomato Passata Puree Gastronomia</t>
+          <t>Mutti Baby Roma Passata Tomato Puree Gastronomia</t>
         </is>
       </c>
       <c r="D113" s="5" t="n">
@@ -11455,14 +11449,14 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/81718/mutti-cherry-tomato-passata-puree-gastronomia</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/81719/mutti-baby-roma-passata-tomato-puree-gastronomia</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>woolworths:81717</t>
+          <t>woolworths:81718</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -11472,20 +11466,20 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Mutti Organic Passata Tomato Puree</t>
+          <t>Mutti Cherry Tomato Passata Puree Gastronomia</t>
         </is>
       </c>
       <c r="D114" s="5" t="n">
-        <v>3.2</v>
+        <v>3.25</v>
       </c>
       <c r="E114" s="5" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="F114" s="5" t="n">
-        <v>3.2</v>
+        <v>3.25</v>
       </c>
       <c r="G114" s="6" t="n">
-        <v>0.3043</v>
+        <v>0.3085</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
@@ -11499,19 +11493,19 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>560g</t>
+          <t>400g</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/81717/mutti-organic-passata-tomato-puree</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/81718/mutti-cherry-tomato-passata-puree-gastronomia</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>woolworths:290301</t>
+          <t>woolworths:81717</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -11521,20 +11515,20 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Mutti Passata Tomato Puree</t>
+          <t>Mutti Organic Passata Tomato Puree</t>
         </is>
       </c>
       <c r="D115" s="5" t="n">
-        <v>2.55</v>
+        <v>3.2</v>
       </c>
       <c r="E115" s="5" t="n">
-        <v>3.7</v>
+        <v>4.6</v>
       </c>
       <c r="F115" s="5" t="n">
-        <v>2.55</v>
+        <v>3.2</v>
       </c>
       <c r="G115" s="6" t="n">
-        <v>0.3108</v>
+        <v>0.3043</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -11548,12 +11542,12 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>560g</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/290301/mutti-passata-tomato-puree</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/81717/mutti-organic-passata-tomato-puree</t>
         </is>
       </c>
     </row>
@@ -11609,7 +11603,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>woolworths:290297</t>
+          <t>woolworths:290301</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -11619,20 +11613,20 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Mutti Passata Tomato Puree With Basil</t>
+          <t>Mutti Passata Tomato Puree</t>
         </is>
       </c>
       <c r="D117" s="5" t="n">
-        <v>3.35</v>
+        <v>2.55</v>
       </c>
       <c r="E117" s="5" t="n">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
       <c r="F117" s="5" t="n">
-        <v>3.35</v>
+        <v>2.55</v>
       </c>
       <c r="G117" s="6" t="n">
-        <v>0.3021</v>
+        <v>0.3108</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
@@ -11646,19 +11640,19 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>700g</t>
+          <t>400g</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/290297/mutti-passata-tomato-puree-with-basil</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/290301/mutti-passata-tomato-puree</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>woolworths:6048427</t>
+          <t>woolworths:218038</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -11668,20 +11662,20 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Mutti Passata Tomato Puree With Basil</t>
+          <t>Mutti Passata Tomato Puree Siciliana</t>
         </is>
       </c>
       <c r="D118" s="5" t="n">
-        <v>2.55</v>
+        <v>3.35</v>
       </c>
       <c r="E118" s="5" t="n">
-        <v>3.7</v>
+        <v>4.8</v>
       </c>
       <c r="F118" s="5" t="n">
-        <v>2.55</v>
+        <v>3.35</v>
       </c>
       <c r="G118" s="6" t="n">
-        <v>0.3108</v>
+        <v>0.3021</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
@@ -11700,221 +11694,233 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6048427/mutti-passata-tomato-puree-with-basil</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/218038/mutti-passata-tomato-puree-siciliana</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
+          <t>woolworths:290297</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Mutti</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Mutti Passata Tomato Puree With Basil</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="E119" s="5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F119" s="5" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="G119" s="6" t="n">
+        <v>0.3021</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>700g</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>https://www.woolworths.com.au/shop/productdetails/290297/mutti-passata-tomato-puree-with-basil</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>woolworths:6048427</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Mutti</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>Mutti Passata Tomato Puree With Basil</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="E120" s="5" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F120" s="5" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="G120" s="6" t="n">
+        <v>0.3108</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>400g</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>https://www.woolworths.com.au/shop/productdetails/6048427/mutti-passata-tomato-puree-with-basil</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
           <t>woolworths:38963</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B121" t="inlineStr">
         <is>
           <t>Val Verde</t>
         </is>
       </c>
-      <c r="C119" s="4" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
         <is>
           <t>Val Verde Passata Sauce</t>
         </is>
       </c>
-      <c r="D119" s="5" t="n">
+      <c r="D121" s="5" t="n">
         <v>3.5</v>
       </c>
-      <c r="E119" s="5" t="n"/>
-      <c r="F119" s="5" t="n"/>
-      <c r="G119" s="6" t="n"/>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr">
+      <c r="E121" s="5" t="n"/>
+      <c r="F121" s="5" t="n"/>
+      <c r="G121" s="6" t="n"/>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr">
+      <c r="J121" t="inlineStr">
         <is>
           <t>700g</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr">
+      <c r="K121" t="inlineStr">
         <is>
           <t>https://www.woolworths.com.au/shop/productdetails/38963/val-verde-passata-sauce</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
         <is>
           <t>Pesto</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="3" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
         <is>
           <t>Product ID</t>
         </is>
       </c>
-      <c r="B122" s="3" t="inlineStr">
+      <c r="B124" s="3" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="C122" s="3" t="inlineStr">
+      <c r="C124" s="3" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="D122" s="3" t="inlineStr">
+      <c r="D124" s="3" t="inlineStr">
         <is>
           <t>Current Price (AUD)</t>
         </is>
       </c>
-      <c r="E122" s="3" t="inlineStr">
+      <c r="E124" s="3" t="inlineStr">
         <is>
           <t>Original Price (AUD)</t>
         </is>
       </c>
-      <c r="F122" s="3" t="inlineStr">
+      <c r="F124" s="3" t="inlineStr">
         <is>
           <t>Promotional Price (AUD)</t>
         </is>
       </c>
-      <c r="G122" s="3" t="inlineStr">
+      <c r="G124" s="3" t="inlineStr">
         <is>
           <t>Discount</t>
         </is>
       </c>
-      <c r="H122" s="3" t="inlineStr">
+      <c r="H124" s="3" t="inlineStr">
         <is>
           <t>Online Only</t>
         </is>
       </c>
-      <c r="I122" s="3" t="inlineStr">
+      <c r="I124" s="3" t="inlineStr">
         <is>
           <t>Availability</t>
         </is>
       </c>
-      <c r="J122" s="3" t="inlineStr">
+      <c r="J124" s="3" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="K122" s="3" t="inlineStr">
+      <c r="K124" s="3" t="inlineStr">
         <is>
           <t>Product URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>woolworths:409785</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>Classic Italia</t>
-        </is>
-      </c>
-      <c r="C123" s="4" t="inlineStr">
-        <is>
-          <t>Classic Italia Green Pesto</t>
-        </is>
-      </c>
-      <c r="D123" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E123" s="5" t="n"/>
-      <c r="F123" s="5" t="n"/>
-      <c r="G123" s="6" t="n"/>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="J123" t="inlineStr">
-        <is>
-          <t>190g</t>
-        </is>
-      </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/409785/classic-italia-green-pesto-190g</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>woolworths:409784</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>Classic Italia</t>
-        </is>
-      </c>
-      <c r="C124" s="4" t="inlineStr">
-        <is>
-          <t>Classic Italia Red Pesto</t>
-        </is>
-      </c>
-      <c r="D124" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E124" s="5" t="n"/>
-      <c r="F124" s="5" t="n"/>
-      <c r="G124" s="6" t="n"/>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>190g</t>
-        </is>
-      </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/409784/classic-italia-red-pesto</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>woolworths:6023657</t>
+          <t>woolworths:409785</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>La Gina</t>
+          <t>Classic Italia</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>La Gina Basil Pesto</t>
+          <t>Classic Italia Green Pesto</t>
         </is>
       </c>
       <c r="D125" s="5" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="E125" s="5" t="n"/>
       <c r="F125" s="5" t="n"/>
@@ -11936,28 +11942,28 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6023657/la-gina-basil-pesto</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/409785/classic-italia-green-pesto-190g</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>woolworths:6023658</t>
+          <t>woolworths:409784</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>La Gina</t>
+          <t>Classic Italia</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>La Gina Sundried Tomato Pesto</t>
+          <t>Classic Italia Red Pesto</t>
         </is>
       </c>
       <c r="D126" s="5" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="E126" s="5" t="n"/>
       <c r="F126" s="5" t="n"/>
@@ -11979,28 +11985,28 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6023658/la-gina-sundried-tomato-pesto</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/409784/classic-italia-red-pesto</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>woolworths:185963</t>
+          <t>woolworths:6023657</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>La Molisana</t>
+          <t>La Gina</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>La Molisana Pesto Al Basilico</t>
+          <t>La Gina Basil Pesto</t>
         </is>
       </c>
       <c r="D127" s="5" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
       <c r="E127" s="5" t="n"/>
       <c r="F127" s="5" t="n"/>
@@ -12022,28 +12028,28 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/185963/la-molisana-pesto-al-basilico</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6023657/la-gina-basil-pesto</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>woolworths:185962</t>
+          <t>woolworths:6023658</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>La Molisana</t>
+          <t>La Gina</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>La Molisana Pesto Rosso</t>
+          <t>La Gina Sundried Tomato Pesto</t>
         </is>
       </c>
       <c r="D128" s="5" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
       <c r="E128" s="5" t="n"/>
       <c r="F128" s="5" t="n"/>
@@ -12065,28 +12071,28 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/185962/la-molisana-pesto-rosso</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6023658/la-gina-sundried-tomato-pesto</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>woolworths:94376</t>
+          <t>woolworths:185963</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Leggo's</t>
+          <t>La Molisana</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Sundried Tomato Red Pesto Sundried Tomato</t>
+          <t>La Molisana Pesto Al Basilico</t>
         </is>
       </c>
       <c r="D129" s="5" t="n">
-        <v>5.3</v>
+        <v>4</v>
       </c>
       <c r="E129" s="5" t="n"/>
       <c r="F129" s="5" t="n"/>
@@ -12108,28 +12114,28 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/94376/leggo-s-sundried-tomato-red-pesto-sundried-tomato</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/185963/la-molisana-pesto-al-basilico</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>woolworths:94375</t>
+          <t>woolworths:185962</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Leggo's</t>
+          <t>La Molisana</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Leggo's Traditional Basil Pesto With Pecorino Cheese</t>
+          <t>La Molisana Pesto Rosso</t>
         </is>
       </c>
       <c r="D130" s="5" t="n">
-        <v>5.3</v>
+        <v>4</v>
       </c>
       <c r="E130" s="5" t="n"/>
       <c r="F130" s="5" t="n"/>
@@ -12151,27 +12157,29 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/94375/leggo-s-traditional-basil-pesto-with-pecorino-cheese</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/185962/la-molisana-pesto-rosso</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>woolworths:6022495</t>
+          <t>woolworths:94376</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Ottolenghi</t>
+          <t>Leggo's</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Ottolenghi Calabrian Chilli &amp; Tomato Pesto Sauce</t>
-        </is>
-      </c>
-      <c r="D131" s="5" t="n"/>
+          <t>Leggo's Sundried Tomato Red Pesto Sundried Tomato</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="n">
+        <v>5.3</v>
+      </c>
       <c r="E131" s="5" t="n"/>
       <c r="F131" s="5" t="n"/>
       <c r="G131" s="6" t="n"/>
@@ -12182,38 +12190,38 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Temporarily unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>170g</t>
+          <t>190g</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6022495/ottolenghi-calabrian-chilli-tomato-pesto-sauce</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/94376/leggo-s-sundried-tomato-red-pesto-sundried-tomato</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>woolworths:55480</t>
+          <t>woolworths:94375</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Ottolenghi</t>
+          <t>Leggo's</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Ottolenghi Miso Pesto</t>
+          <t>Leggo's Traditional Basil Pesto With Pecorino Cheese</t>
         </is>
       </c>
       <c r="D132" s="5" t="n">
-        <v>13</v>
+        <v>5.3</v>
       </c>
       <c r="E132" s="5" t="n"/>
       <c r="F132" s="5" t="n"/>
@@ -12230,42 +12238,44 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>170g</t>
+          <t>190g</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/55480/ottolenghi-miso-pesto</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/94375/leggo-s-traditional-basil-pesto-with-pecorino-cheese</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>woolworths:6059196</t>
+          <t>woolworths:876758</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Providore</t>
+          <t>Lucia's</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Providore Italian Basil Pecorino &amp; Pine Nut Pesto</t>
+          <t>Lucia's Artichoke &amp; Pistachio Pesto</t>
         </is>
       </c>
       <c r="D133" s="5" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="E133" s="5" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F133" s="5" t="n">
-        <v>5.5</v>
+        <v>8</v>
+      </c>
+      <c r="F133" s="5" t="inlineStr">
+        <is>
+          <t>2 for $14.00</t>
+        </is>
       </c>
       <c r="G133" s="6" t="n">
-        <v>0.1538</v>
+        <v>0.125</v>
       </c>
       <c r="H133" t="inlineStr">
         <is>
@@ -12284,37 +12294,39 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6059196/providore-italian-basil-pecorino-pine-nut-pesto</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/876758/lucia-s-artichoke-pistachio-pesto</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>woolworths:947979</t>
+          <t>woolworths:882049</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Roza's</t>
+          <t>Lucia's</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Roza's Traditional Pesto</t>
+          <t>Lucia's Basil Pesto</t>
         </is>
       </c>
       <c r="D134" s="5" t="n">
-        <v>6.8</v>
+        <v>8</v>
       </c>
       <c r="E134" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F134" s="5" t="n">
-        <v>6.8</v>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>2 for $14.00</t>
+        </is>
       </c>
       <c r="G134" s="6" t="n">
-        <v>0.15</v>
+        <v>0.125</v>
       </c>
       <c r="H134" t="inlineStr">
         <is>
@@ -12328,37 +12340,45 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>200mL</t>
+          <t>190g</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/947979/roza-s-traditional-pesto</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/882049/lucia-s-basil-pesto</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>woolworths:34565</t>
+          <t>woolworths:882262</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Sacla</t>
+          <t>Lucia's</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Sacla Classic Basil Pesto</t>
+          <t>Lucia's Sundried Tomato Pesto</t>
         </is>
       </c>
       <c r="D135" s="5" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="E135" s="5" t="n"/>
-      <c r="F135" s="5" t="n"/>
-      <c r="G135" s="6" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="E135" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F135" s="5" t="inlineStr">
+        <is>
+          <t>2 for $14.00</t>
+        </is>
+      </c>
+      <c r="G135" s="6" t="n">
+        <v>0.125</v>
+      </c>
       <c r="H135" t="inlineStr">
         <is>
           <t>No</t>
@@ -12376,28 +12396,28 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/34565/sacla-classic-basil-pesto</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/882262/lucia-s-sundried-tomato-pesto</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>woolworths:88376</t>
+          <t>woolworths:6022495</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Sacla</t>
+          <t>Ottolenghi</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Sacla Tomato Pesto Free From</t>
+          <t>Ottolenghi Calabrian Chilli &amp; Tomato Pesto Sauce</t>
         </is>
       </c>
       <c r="D136" s="5" t="n">
-        <v>5.3</v>
+        <v>13</v>
       </c>
       <c r="E136" s="5" t="n"/>
       <c r="F136" s="5" t="n"/>
@@ -12414,37 +12434,43 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>190g</t>
+          <t>170g</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/88376/sacla-tomato-pesto-free-from</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6022495/ottolenghi-calabrian-chilli-tomato-pesto-sauce</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>woolworths:385698</t>
+          <t>woolworths:6059196</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Woolworths</t>
+          <t>Providore</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Woolworths Basil Pesto Pasta Salad</t>
+          <t>Providore Italian Basil Pecorino &amp; Pine Nut Pesto</t>
         </is>
       </c>
       <c r="D137" s="5" t="n">
         <v>5.5</v>
       </c>
-      <c r="E137" s="5" t="n"/>
-      <c r="F137" s="5" t="n"/>
-      <c r="G137" s="6" t="n"/>
+      <c r="E137" s="5" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F137" s="5" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G137" s="6" t="n">
+        <v>0.1538</v>
+      </c>
       <c r="H137" t="inlineStr">
         <is>
           <t>No</t>
@@ -12457,33 +12483,33 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>250g</t>
+          <t>190g</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/385698/woolworths-basil-pesto-pasta-salad</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6059196/providore-italian-basil-pecorino-pine-nut-pesto</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>woolworths:294743</t>
+          <t>woolworths:34565</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Woolworths</t>
+          <t>Sacla</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Woolworths Basil Pesto Pasta Salad Kit</t>
+          <t>Sacla Classic Basil Pesto</t>
         </is>
       </c>
       <c r="D138" s="5" t="n">
-        <v>9.9</v>
+        <v>5.3</v>
       </c>
       <c r="E138" s="5" t="n"/>
       <c r="F138" s="5" t="n"/>
@@ -12500,33 +12526,33 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>400g</t>
+          <t>190g</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/294743/woolworths-basil-pesto-pasta-salad-kit</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/34565/sacla-classic-basil-pesto</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>woolworths:6050785</t>
+          <t>woolworths:88376</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Woolworths</t>
+          <t>Sacla</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Woolworths Chicken Pesto Pasta Bake</t>
+          <t>Sacla Tomato Pesto Free From</t>
         </is>
       </c>
       <c r="D139" s="5" t="n">
-        <v>8.5</v>
+        <v>5.3</v>
       </c>
       <c r="E139" s="5" t="n"/>
       <c r="F139" s="5" t="n"/>
@@ -12543,37 +12569,43 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>350g</t>
+          <t>190g</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6050785/woolworths-chicken-pesto-pasta-bake</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/88376/sacla-tomato-pesto-free-from</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>woolworths:6051249</t>
+          <t>woolworths:6041658</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Woolworths</t>
+          <t>Strength Meals Co</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Woolworths Creamy Tomato &amp; Pesto Chicken Pasta Bake</t>
+          <t>Strength Meals Co Chicken Pesto Pasta Salad</t>
         </is>
       </c>
       <c r="D140" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="E140" s="5" t="n"/>
-      <c r="F140" s="5" t="n"/>
-      <c r="G140" s="6" t="n"/>
+        <v>9</v>
+      </c>
+      <c r="E140" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F140" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G140" s="6" t="n">
+        <v>0.1</v>
+      </c>
       <c r="H140" t="inlineStr">
         <is>
           <t>No</t>
@@ -12586,19 +12618,19 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>1.3kg</t>
+          <t>340g</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>https://www.woolworths.com.au/shop/productdetails/6051249/woolworths-creamy-tomato-pesto-chicken-pasta-bake</t>
+          <t>https://www.woolworths.com.au/shop/productdetails/6041658/strength-meals-co-chicken-pesto-pasta-salad</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>woolworths:753340</t>
+          <t>woolworths:385698</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -12608,11 +12640,11 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Woolworths Pesto Basil</t>
+          <t>Woolworths Basil Pesto Pasta Salad</t>
         </is>
       </c>
       <c r="D141" s="5" t="n">
-        <v>1.95</v>
+        <v>5.5</v>
       </c>
       <c r="E141" s="5" t="n"/>
       <c r="F141" s="5" t="n"/>
@@ -12629,10 +12661,147 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>https://www.woolworths.com.au/shop/productdetails/385698/woolworths-basil-pesto-pasta-salad</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>woolworths:294743</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Woolworths</t>
+        </is>
+      </c>
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>Woolworths Basil Pesto Pasta Salad Kit</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E142" s="5" t="n"/>
+      <c r="F142" s="5" t="n"/>
+      <c r="G142" s="6" t="n"/>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>400g</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>https://www.woolworths.com.au/shop/productdetails/294743/woolworths-basil-pesto-pasta-salad-kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>woolworths:6050785</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Woolworths</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>Woolworths Chicken Pesto Pasta Bake</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E143" s="5" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>2 for $16.00</t>
+        </is>
+      </c>
+      <c r="G143" s="6" t="n">
+        <v>0.0588</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>350g</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>https://www.woolworths.com.au/shop/productdetails/6050785/woolworths-chicken-pesto-pasta-bake</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>woolworths:753340</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Woolworths</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>Woolworths Pesto Basil</t>
+        </is>
+      </c>
+      <c r="D144" s="5" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="E144" s="5" t="n"/>
+      <c r="F144" s="5" t="n"/>
+      <c r="G144" s="6" t="n"/>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
           <t>190g</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr">
+      <c r="K144" t="inlineStr">
         <is>
           <t>https://www.woolworths.com.au/shop/productdetails/753340/woolworths-pesto-basil</t>
         </is>
@@ -12642,8 +12811,8 @@
   <mergeCells count="5">
     <mergeCell ref="A100:K100"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="A121:K121"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="A123:K123"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <hyperlinks>
@@ -12665,7 +12834,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId22"/>
@@ -12756,8 +12925,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId114"/>
@@ -12775,13 +12944,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId131"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="4">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId129"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId130"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId131"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId132"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId133"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId134"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId135"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12901,7 +13073,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -12959,7 +13131,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -13023,7 +13195,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -13203,7 +13375,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -13261,7 +13433,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -13325,7 +13497,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -13801,7 +13973,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -13923,7 +14095,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -14271,7 +14443,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -14329,7 +14501,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -14445,7 +14617,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -14509,7 +14681,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -14573,7 +14745,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -14811,7 +14983,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -14869,7 +15041,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -14933,7 +15105,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -14997,7 +15169,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -15061,7 +15233,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -15485,7 +15657,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -15601,7 +15773,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -15665,7 +15837,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -16199,7 +16371,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
@@ -16605,7 +16777,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
@@ -16727,7 +16899,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -16791,7 +16963,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
@@ -16855,7 +17027,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
@@ -16977,7 +17149,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
@@ -17035,7 +17207,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -17985,7 +18157,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
@@ -18165,7 +18337,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
@@ -18223,7 +18395,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
@@ -18287,7 +18459,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
@@ -18351,7 +18523,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
@@ -18415,7 +18587,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
@@ -18479,7 +18651,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
@@ -18537,7 +18709,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
@@ -18601,7 +18773,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
@@ -18723,7 +18895,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
@@ -18787,7 +18959,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
@@ -18851,7 +19023,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
@@ -18915,7 +19087,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E103" s="4" t="inlineStr">
@@ -19037,7 +19209,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E105" s="4" t="inlineStr">
@@ -19159,7 +19331,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E107" s="4" t="inlineStr">
@@ -19275,7 +19447,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E109" s="4" t="inlineStr">
@@ -19397,7 +19569,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E111" s="4" t="inlineStr">
@@ -19577,7 +19749,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
@@ -19699,7 +19871,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
@@ -19763,7 +19935,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E117" s="4" t="inlineStr">
@@ -19999,7 +20171,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E121" s="4" t="inlineStr">
@@ -20063,7 +20235,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
@@ -20127,7 +20299,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E123" s="4" t="inlineStr">
@@ -20191,7 +20363,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
@@ -20255,7 +20427,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E125" s="4" t="inlineStr">
@@ -20319,7 +20491,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
@@ -20383,7 +20555,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E127" s="4" t="inlineStr">
@@ -20563,7 +20735,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
@@ -20807,7 +20979,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
@@ -20865,7 +21037,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E135" s="4" t="inlineStr">
@@ -20923,7 +21095,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
@@ -20981,7 +21153,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E137" s="4" t="inlineStr">
@@ -21039,7 +21211,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E138" s="4" t="inlineStr">
@@ -21097,7 +21269,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E139" s="4" t="inlineStr">
@@ -21161,7 +21333,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
@@ -21225,7 +21397,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E141" s="4" t="inlineStr">
@@ -21289,7 +21461,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
@@ -21353,7 +21525,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E143" s="4" t="inlineStr">
@@ -21417,7 +21589,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
@@ -21481,7 +21653,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E145" s="4" t="inlineStr">
@@ -21545,7 +21717,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
@@ -21609,7 +21781,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E147" s="4" t="inlineStr">
@@ -21795,7 +21967,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
@@ -22039,7 +22211,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
@@ -22103,7 +22275,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Price changed; Original price changed; Promotional price changed; Discount percentage changed</t>
+          <t>Price changed</t>
         </is>
       </c>
       <c r="E155" s="4" t="inlineStr">

</xml_diff>